<commit_message>
Agregar barra filtro en despachos
</commit_message>
<xml_diff>
--- a/Formatos/Formato SOLPED.xlsx
+++ b/Formatos/Formato SOLPED.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Python\Proyecto Control QP\Formatos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{70932A01-E3DC-4085-B8BC-7992DE0EE6AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD628E91-B330-40CC-8D25-11A19026AA75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{05E38F80-7958-4879-911A-47BE11C226FD}"/>
   </bookViews>
@@ -34,42 +34,66 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>Tienda</t>
   </si>
   <si>
-    <t>Tienda1</t>
-  </si>
-  <si>
-    <t>Tienda2</t>
-  </si>
-  <si>
-    <t>Tienda3</t>
-  </si>
-  <si>
-    <t>Tienda4</t>
-  </si>
-  <si>
-    <t>Tienda5</t>
-  </si>
-  <si>
-    <t>Producto1</t>
-  </si>
-  <si>
-    <t>Producto2</t>
-  </si>
-  <si>
-    <t>Producto3</t>
-  </si>
-  <si>
-    <t>Producto4</t>
-  </si>
-  <si>
-    <t>Producto5</t>
-  </si>
-  <si>
     <t>FECHA DE DESPACHO:</t>
+  </si>
+  <si>
+    <t>PVEA SALAVERRY</t>
+  </si>
+  <si>
+    <t>PVEA SUCRE</t>
+  </si>
+  <si>
+    <t>PVEA CALLAO</t>
+  </si>
+  <si>
+    <t>PVEA SAN BORJA</t>
+  </si>
+  <si>
+    <t>PVEA MIRAFLORES</t>
+  </si>
+  <si>
+    <t>PVEA AREQUIPA</t>
+  </si>
+  <si>
+    <t>PVEA TRUJILLO</t>
+  </si>
+  <si>
+    <t>PVEA CHICLAYO</t>
+  </si>
+  <si>
+    <t>PVEA PIURA</t>
+  </si>
+  <si>
+    <t>PVEA CHIMBOTE</t>
+  </si>
+  <si>
+    <t>HEY FIT TORONJA</t>
+  </si>
+  <si>
+    <t>HEY FIT PIÑA</t>
+  </si>
+  <si>
+    <t>HEY FIT GOLDEN</t>
+  </si>
+  <si>
+    <t>COOLER ROJO</t>
+  </si>
+  <si>
+    <t>VASOS 5 OZ</t>
+  </si>
+  <si>
+    <t>POLO</t>
+  </si>
+  <si>
+    <t>FALDA</t>
+  </si>
+  <si>
+    <t>GORRA</t>
   </si>
 </sst>
 </file>
@@ -608,11 +632,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D970FE4-8C3A-4D4C-A75D-55965E814938}">
-  <dimension ref="A1:AJ9"/>
+  <dimension ref="A1:AJ14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" customWidth="1"/>
-    <col min="5" max="36" width="11.5546875" style="3"/>
+    <col min="3" max="3" width="5.44140625" customWidth="1"/>
+    <col min="4" max="4" width="22.44140625" customWidth="1"/>
+    <col min="5" max="12" width="15.77734375" style="3" customWidth="1"/>
+    <col min="13" max="36" width="11.5546875" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="26.4" customHeight="1" x14ac:dyDescent="0.3"/>
@@ -620,32 +647,38 @@
     <row r="3" spans="1:21" ht="35.4" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="B4" s="1">
-        <v>46233</v>
+        <v>46240</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>0</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="I4" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="J4" s="5"/>
-      <c r="K4" s="5"/>
-      <c r="L4" s="5"/>
+        <v>16</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="L4" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="M4" s="5"/>
       <c r="N4" s="5"/>
       <c r="O4" s="5"/>
@@ -658,78 +691,294 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="D5" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="3">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="F5" s="3">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="G5" s="3">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="H5" s="3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I5" s="3">
-        <v>10</v>
+        <v>200</v>
+      </c>
+      <c r="J5" s="3">
+        <v>1</v>
+      </c>
+      <c r="K5" s="3">
+        <v>1</v>
+      </c>
+      <c r="L5" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.3">
       <c r="D6" t="s">
-        <v>2</v>
+        <v>3</v>
+      </c>
+      <c r="E6" s="3">
+        <v>24</v>
+      </c>
+      <c r="F6" s="3">
+        <v>24</v>
       </c>
       <c r="G6" s="3">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="H6" s="3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I6" s="3">
-        <v>10</v>
+        <v>200</v>
+      </c>
+      <c r="J6" s="3">
+        <v>1</v>
+      </c>
+      <c r="K6" s="3">
+        <v>1</v>
+      </c>
+      <c r="L6" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="D7" t="s">
-        <v>3</v>
+        <v>4</v>
+      </c>
+      <c r="E7" s="3">
+        <v>24</v>
+      </c>
+      <c r="F7" s="3">
+        <v>24</v>
       </c>
       <c r="G7" s="3">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="H7" s="3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I7" s="3">
-        <v>10</v>
+        <v>200</v>
+      </c>
+      <c r="J7" s="3">
+        <v>1</v>
+      </c>
+      <c r="K7" s="3">
+        <v>1</v>
+      </c>
+      <c r="L7" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="D8" t="s">
-        <v>4</v>
+        <v>5</v>
+      </c>
+      <c r="E8" s="3">
+        <v>24</v>
+      </c>
+      <c r="F8" s="3">
+        <v>24</v>
       </c>
       <c r="G8" s="3">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="H8" s="3">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="I8" s="3">
-        <v>10</v>
+        <v>200</v>
+      </c>
+      <c r="J8" s="3">
+        <v>1</v>
+      </c>
+      <c r="K8" s="3">
+        <v>1</v>
+      </c>
+      <c r="L8" s="3">
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.3">
       <c r="D9" t="s">
-        <v>5</v>
+        <v>6</v>
+      </c>
+      <c r="E9" s="3">
+        <v>24</v>
+      </c>
+      <c r="F9" s="3">
+        <v>24</v>
       </c>
       <c r="G9" s="3">
+        <v>24</v>
+      </c>
+      <c r="H9" s="3">
+        <v>1</v>
+      </c>
+      <c r="I9" s="3">
+        <v>200</v>
+      </c>
+      <c r="J9" s="3">
+        <v>1</v>
+      </c>
+      <c r="K9" s="3">
+        <v>1</v>
+      </c>
+      <c r="L9" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="3">
+        <v>24</v>
+      </c>
+      <c r="F10" s="3">
+        <v>24</v>
+      </c>
+      <c r="G10" s="3">
+        <v>24</v>
+      </c>
+      <c r="H10" s="3">
+        <v>1</v>
+      </c>
+      <c r="I10" s="3">
+        <v>200</v>
+      </c>
+      <c r="J10" s="3">
+        <v>1</v>
+      </c>
+      <c r="K10" s="3">
+        <v>1</v>
+      </c>
+      <c r="L10" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="3">
+        <v>24</v>
+      </c>
+      <c r="F11" s="3">
+        <v>24</v>
+      </c>
+      <c r="G11" s="3">
+        <v>24</v>
+      </c>
+      <c r="H11" s="3">
+        <v>1</v>
+      </c>
+      <c r="I11" s="3">
+        <v>200</v>
+      </c>
+      <c r="J11" s="3">
+        <v>1</v>
+      </c>
+      <c r="K11" s="3">
+        <v>1</v>
+      </c>
+      <c r="L11" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="D12" t="s">
+        <v>9</v>
+      </c>
+      <c r="E12" s="3">
+        <v>24</v>
+      </c>
+      <c r="F12" s="3">
+        <v>24</v>
+      </c>
+      <c r="G12" s="3">
+        <v>24</v>
+      </c>
+      <c r="H12" s="3">
+        <v>1</v>
+      </c>
+      <c r="I12" s="3">
+        <v>200</v>
+      </c>
+      <c r="J12" s="3">
+        <v>1</v>
+      </c>
+      <c r="K12" s="3">
+        <v>1</v>
+      </c>
+      <c r="L12" s="3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="D13" t="s">
         <v>10</v>
       </c>
-      <c r="H9" s="3">
-        <v>5</v>
-      </c>
-      <c r="I9" s="3">
-        <v>10</v>
+      <c r="E13" s="3">
+        <v>24</v>
+      </c>
+      <c r="F13" s="3">
+        <v>24</v>
+      </c>
+      <c r="G13" s="3">
+        <v>24</v>
+      </c>
+      <c r="H13" s="3">
+        <v>1</v>
+      </c>
+      <c r="I13" s="3">
+        <v>200</v>
+      </c>
+      <c r="J13" s="3">
+        <v>1</v>
+      </c>
+      <c r="K13" s="3">
+        <v>1</v>
+      </c>
+      <c r="L13" s="3">
+        <v>1</v>
+      </c>
+      <c r="R13"/>
+      <c r="S13"/>
+    </row>
+    <row r="14" spans="1:21" x14ac:dyDescent="0.3">
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="3">
+        <v>24</v>
+      </c>
+      <c r="F14" s="3">
+        <v>24</v>
+      </c>
+      <c r="G14" s="3">
+        <v>24</v>
+      </c>
+      <c r="H14" s="3">
+        <v>1</v>
+      </c>
+      <c r="I14" s="3">
+        <v>200</v>
+      </c>
+      <c r="J14" s="3">
+        <v>1</v>
+      </c>
+      <c r="K14" s="3">
+        <v>1</v>
+      </c>
+      <c r="L14" s="3">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>